<commit_message>
feat(F-NAR-019): ATOM-AUT.RAN.001-01 La nappe à carreaux
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.RAN.001-01.xlsx
+++ b/stories/arbres/ATOM-AUT.RAN.001-01.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Raphaël veut le gâteau sur la nappe à carreaux, avec son doudou. La tour recouvre le doudou. Il met les cubes dans la caisse pour voir dessous. Le doudou apparaît. Ils goûtent.</t>
+          <t>La vanille arrive dans le salon, avant le gâteau. Sur un carreau rouge, un éclat de nappe brille. Raphaël veut la tour haute, maintenant, avec le doudou. Un cube glisse : le doudou disparaît. Il cherche sous la nappe, sous le coussin, puis prend toute la pile : les cubes s'éparpillent. Il refuse de foncer, pose un cube, retrouve le doudou. Sur la nappe ouverte, l'éclat de nappe tient au carreau du doudou.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La cuillère en bois tape dans le bol. Ça sent la vanille, tout chaud. Une buée perle sur la vitre. Une goutte glisse, tout doucement. Le gâteau est bientôt prêt. Il sent bon, papa. Dans le salon, le tapis est épais. Une nappe à carreaux attend. Elle est encore pliée, sur la chaise. Le tissu sent un peu le savon. En ce moment, Raphaël est là. Des cubes verts attendent. Des cubes jaunes aussi. Je fais une tour, maman. Pendant que le gâteau refroidit ? Oui, une tour haute. Raphaël pose un cube vert. Clic. Puis un cube jaune. Clic. La tour grandit au milieu. Elle est belle, ta tour. Le cube du haut, c'est le gâteau. Un gâteau de cubes ! Le doudou gris est au pied. Raphaël l'assoit contre la tour. Toi, tu goûtes avec nous. Il pose encore un cube. Clic. Un cube jaune glisse. La tour penche un peu. Trois cubes tombent sur le doudou. Oh. Ça a bougé. Raphaël cherche du regard. Où est mon doudou ? Sur la chaise, peut-être ? Il va vers la chaise. La nappe est là, seule. Pas de tissu gris. Sous la nappe ? Il soulève un coin doux. Rien. Près du canapé ? Sa main passe sous le coussin. Le coussin est moelleux. Le doudou n'est pas là. Il est perdu. La tour est encore au milieu. Le tapis disparaît sous les cubes. Je veux voir dessous. Raphaël prend le cube du haut. Il le pose dans la caisse. Toc. Le bois sent un peu la forêt.</t>
+          <t>La vanille arrive dans le salon, avant le gâteau. Un carré de buée s'ouvre sur la vitre. La cuillère en bois tape dans le bol. Le gâteau est bientôt prêt. Il sent bon, papa. Dans le salon, le tapis est épais. Une nappe à carreaux attend, pliée. Elle repose sur la chaise. Sur un carreau rouge, un éclat de nappe brille. Il est tout petit, maman. C'est un éclat de nappe. Le tissu sent un peu le savon. Raphaël, tu sens le gâteau ? Oui, papa. Je veux la tour, maintenant ! Pendant que le gâteau refroidit ? Oui, une tour haute. En ce moment, Raphaël saisit un cube. Le cube vert est lisse, un peu froid. Il le pose au milieu du tapis. Ça fait clic, tout petit. Puis un cube jaune. Ça fait clic, contre le vert. Le cube du haut, c'est le gâteau. Un gâteau de cubes ! Le doudou gris est au pied. Raphaël l'assoit contre la tour. Toi, tu goûtes avec nous. Elle est belle, ta tour. Raphaël veut un cube de plus. Il le pose trop vite. Un cube jaune glisse. La tour penche. Trois cubes tombent sur le doudou. Oh. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Où est mon doudou ? Sous la nappe, peut-être ? Il va vers la chaise. Il soulève un coin du tissu. L'éclat de nappe tremble, puis tient. Pas de tissu gris. Il n'est pas là. Près du canapé ? Sa main passe sous le coussin. Le coussin est moelleux. Le doudou n'est pas là. Il est perdu. Je prends tout, d'un coup ! Il saisit la pile trop vite. Les cubes glissent entre ses doigts. Le tapis disparaît sous les cubes. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes sous les cubes ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La cuillère en bois tape dans le bol. Ça sent la vanille, tout chaud. Une buée perle sur la vitre. Une goutte glisse, tout doucement. Le gâteau est bientôt prêt. Il sent bon, papa. Dans le salon, le tapis est épais. Une nappe à carreaux attend. Elle est encore pliée, sur la chaise. Le tissu sent un peu le savon. En ce moment, Raphaël est là. Des cubes verts attendent. Des cubes jaunes aussi. Je fais une tour, maman. Pendant que le gâteau refroidit ? Oui, une tour haute. Raphaël pose un cube vert. Clic. Puis un cube jaune. Clic. La tour grandit au milieu. Elle est belle, ta tour. Le cube du haut, c'est le gâteau. Un gâteau de cubes ! Le doudou gris est au pied. Raphaël l'assoit contre la tour. Toi, tu goûtes avec nous. Il pose encore un cube. Clic. Un cube jaune glisse. La tour penche un peu. Trois cubes tombent sur le doudou. Oh. Ça a bougé. Raphaël cherche du regard. Où est mon doudou ? Sur la chaise, peut-être ? Il va vers la chaise. La nappe est là, seule. Pas de tissu gris. Sous la nappe ? Il soulève un coin doux. Rien. Près du canapé ? Sa main passe sous le coussin. Le coussin est moelleux. Le doudou n'est pas là. Il est perdu. La tour est encore au milieu. Le tapis disparaît sous les cubes. Je veux voir dessous. Raphaël prend le cube du haut. Il le pose dans la caisse. Toc. Le bois sent un peu la forêt.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La vanille arrive dans le salon, avant le gâteau. Un carré de buée s'ouvre sur la vitre. La cuillère en bois tape dans le bol. Le gâteau est bientôt prêt. Il sent bon, papa. Dans le salon, le tapis est épais. Une nappe à carreaux attend, pliée. Elle repose sur la chaise. Sur un carreau rouge, un &lt;emphasis level="moderate"&gt;éclat de nappe&lt;/emphasis&gt; brille. Il est tout petit, maman. C'est un éclat de nappe. Le tissu sent un peu le savon. Raphaël, tu sens le gâteau ? Oui, papa. Je veux la tour, maintenant ! Pendant que le gâteau refroidit ? Oui, une tour haute. En ce moment, Raphaël saisit un cube. Le cube vert est lisse, un peu froid. Il le pose au milieu du tapis. Ça fait clic, tout petit. Puis un cube jaune. Ça fait clic, contre le vert. Le cube du haut, c'est le gâteau. Un gâteau de cubes ! Le doudou gris est au pied. Raphaël l'assoit contre la tour. Toi, tu goûtes avec nous. Elle est belle, ta tour. Raphaël veut un cube de plus. Il le pose trop vite. Un cube jaune glisse. La tour penche. Trois cubes tombent sur le doudou. Oh. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Où est mon doudou ? Sous la nappe, peut-être ? Il va vers la chaise. Il soulève un coin du tissu. L'éclat de nappe tremble, puis tient. Pas de tissu gris. Il n'est pas là. Près du canapé ? Sa main passe sous le coussin. Le coussin est moelleux. Le doudou n'est pas là. Il est perdu. Je prends tout, d'un coup ! Il saisit la pile trop vite. Les cubes glissent entre ses doigts. Le tapis disparaît sous les cubes. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes sous les cubes ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Léa joue dans le salon. Maman est sur le canapé. Léa a des cubes. Les cubes sont verts et jaunes. Léa fait une tour. La tour est haute. Les cubes font clic. Puis le jeu est fini. Maman dit : c'est l'heure de &lt;emphasis&gt;ranger&lt;/emphasis&gt;. Léa prend un cube. Elle le met dans la caisse. Elle prend un autre cube. Elle le met dans la caisse. Encore un cube. Dans la caisse. La caisse est pleine. Le tapis est vide. Ranger, c'est mettre dans la caisse. Maman dit : merci Léa.&lt;/slow&gt; [pause]</t>
+          <t>La vanille arrive dans le salon, avant le gâteau. Un carré de buée s'ouvre sur la vitre. La cuillère en bois tape dans le bol. Le gâteau est bientôt prêt. Il sent bon, papa. Dans le salon, le tapis est épais. Une nappe à carreaux attend, pliée. Elle repose sur la chaise. Sur un carreau rouge, un &lt;emphasis&gt;éclat de nappe&lt;/emphasis&gt; brille. Il est tout petit, maman. C'est un éclat de nappe. Le tissu sent un peu le savon. Raphaël, tu sens le gâteau ? Oui, papa. Je veux la tour, maintenant ! Pendant que le gâteau refroidit ? Oui, une tour haute. En ce moment, Raphaël saisit un cube. Le cube vert est lisse, un peu froid. Il le pose au milieu du tapis. Ça fait clic, tout petit. Puis un cube jaune. Ça fait clic, contre le vert. Le cube du haut, c'est le gâteau. Un gâteau de cubes ! Le doudou gris est au pied. Raphaël l'assoit contre la tour. Toi, tu goûtes avec nous. Elle est belle, ta tour. Raphaël veut un cube de plus. Il le pose trop vite. Un cube jaune glisse. La tour penche. Trois cubes tombent sur le doudou. Oh. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Où est mon doudou ? Sous la nappe, peut-être ? Il va vers la chaise. Il soulève un coin du tissu. L'éclat de nappe tremble, puis tient. Pas de tissu gris. Il n'est pas là. Près du canapé ? Sa main passe sous le coussin. Le coussin est moelleux. Le doudou n'est pas là. Il est perdu. Je prends tout, d'un coup ! Il saisit la pile trop vite. Les cubes glissent entre ses doigts. Le tapis disparaît sous les cubes. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes sous les cubes ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>ranger</t>
+          <t>éclat de nappe</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,66 +1319,77 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_la_tour_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La cuillère en bois tape dans le bol.
-narrateur|Ça sent la vanille, tout chaud.
-narrateur|Une buée perle sur la vitre.
-narrateur|Une goutte glisse, tout doucement.
+          <t>narrateur|La vanille arrive dans le salon, avant le gâteau.
+narrateur|Un carré de buée s'ouvre sur la vitre.
+narrateur|La cuillère en bois tape dans le bol.
 papa|Le gâteau est bientôt prêt.
 maman|Il sent bon, papa.
 narrateur|Dans le salon, le tapis est épais.
-narrateur|Une nappe à carreaux attend.
-narrateur|Elle est encore pliée, sur la chaise.
+narrateur|Une nappe à carreaux attend, pliée.
+narrateur|Elle repose sur la chaise.
+narrateur|Sur un carreau rouge, un éclat de nappe brille.
+enfant-m|Il est tout petit, maman.
+maman|C'est un éclat de nappe.
 narrateur|Le tissu sent un peu le savon.
-narrateur|En ce moment, Raphaël est là.
-narrateur|Des cubes verts attendent.
-narrateur|Des cubes jaunes aussi.
-enfant-m|Je fais une tour, maman.
+papa|Raphaël, tu sens le gâteau ?
+enfant-m|Oui, papa.
+enfant-m|Je veux la tour, maintenant !
 maman|Pendant que le gâteau refroidit ?
 enfant-m|Oui, une tour haute.
-narrateur|Raphaël pose un cube vert.
-narrateur|Clic.
+narrateur|En ce moment, Raphaël saisit un cube.
+narrateur|Le cube vert est lisse, un peu froid.
+narrateur|Il le pose au milieu du tapis.
+narrateur|Ça fait clic, tout petit.
 narrateur|Puis un cube jaune.
-narrateur|Clic.
-narrateur|La tour grandit au milieu.
-papa|Elle est belle, ta tour.
+narrateur|Ça fait clic, contre le vert.
 enfant-m|Le cube du haut, c'est le gâteau.
 maman|Un gâteau de cubes !
 narrateur|Le doudou gris est au pied.
 narrateur|Raphaël l'assoit contre la tour.
 enfant-m|Toi, tu goûtes avec nous.
-narrateur|Il pose encore un cube.
-narrateur|Clic.
+papa|Elle est belle, ta tour.
+narrateur|Raphaël veut un cube de plus.
+narrateur|Il le pose trop vite.
 narrateur|Un cube jaune glisse.
-narrateur|La tour penche un peu.
+narrateur|La tour penche.
 narrateur|Trois cubes tombent sur le doudou.
 enfant-m|Oh.
-papa|Ça a bougé.
-narrateur|Raphaël cherche du regard.
+narrateur|Le sourire de Raphaël disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
 enfant-m|Où est mon doudou ?
-maman|Sur la chaise, peut-être ?
+maman|Sous la nappe, peut-être ?
 narrateur|Il va vers la chaise.
-narrateur|La nappe est là, seule.
+narrateur|Il soulève un coin du tissu.
+narrateur|L'éclat de nappe tremble, puis tient.
 narrateur|Pas de tissu gris.
-enfant-m|Sous la nappe ?
-narrateur|Il soulève un coin doux.
-narrateur|Rien.
+enfant-m|Il n'est pas là.
 papa|Près du canapé ?
 narrateur|Sa main passe sous le coussin.
 narrateur|Le coussin est moelleux.
 narrateur|Le doudou n'est pas là.
 enfant-m|Il est perdu.
-maman|La tour est encore au milieu.
+enfant-m|Je prends tout, d'un coup !
+narrateur|Il saisit la pile trop vite.
+narrateur|Les cubes glissent entre ses doigts.
 narrateur|Le tapis disparaît sous les cubes.
-enfant-m|Je veux voir dessous.
-narrateur|Raphaël prend le cube du haut.
-narrateur|Il le pose dans la caisse.
-narrateur|Toc.
-narrateur|Le bois sent un peu la forêt.</t>
+enfant-m|Ça ne veut pas, papa.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa se baisse à sa hauteur.
+papa|Tu regardes sous les cubes ?</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>cuillère,cubes</t>
         </is>
       </c>
     </row>
@@ -1410,12 +1421,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Raphaël cherche son doudou. Où est-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Raphaël cherche son &lt;emphasis level="moderate"&gt;doudou&lt;/emphasis&gt;. Où est-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Après le jeu, que fait Léa ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Raphaël cherche son &lt;emphasis&gt;doudou&lt;/emphasis&gt;. Où est-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1478,7 +1489,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1486,10 +1497,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1504,34 +1515,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>doudou</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1540,13 +1555,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1556,7 +1571,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=le_doudou_est_sous_les_cubes; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1589,17 +1604,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Un cube vert reste sur le tapis. Raphaël le glisse dans la caisse. Toc. Tu regardes bien dessous ? Oui, maman. La tour devient plus petite. Un bout de tapis reparaît. Encore un, tout doux. Le cube jaune va dans la caisse. Toc. Raphaël écarte un cube bas. Un coin de tissu gris. Mon doudou ! Le doudou était sous la tour. Il sent encore le lit. Raphaël le serre contre sa joue. Le tissu est chaud, tout doux. Te voilà, petit. Merci, tu l'as trouvé. Il était dessous. La caisse a presque tous les cubes. Le tapis est libre, au milieu. La nappe peut s'ouvrir, maintenant.</t>
+          <t>Raphaël refuse de prendre toute la pile. Il pose un genou au tapis. Un cube vert reste près de sa main. Je le mets tout seul. Il glisse le cube dans la caisse. Toc. Le bois sent un peu la forêt. Tu regardes bien dessous ? Oui, maman. La tour devient plus petite. Un bout de tapis reparaît. Le cube jaune va dans la caisse. Toc. Je sors le reste, d'un coup ! Il tire trop fort sur un cube bas. Deux cubes retombent, comme un toit. Oh. Il ne reprend pas trop vite. Il écoute le salon, un instant. Sur la chaise, l'éclat de nappe brille. Il est là. Raphaël refuse de foncer. Il écarte un cube, lentement. Un coin de tissu gris. Mon doudou ! Le doudou était sous la tour. Il sent le tapis, un peu chaud. Raphaël le serre contre sa joue. Merci, Raphaël. Il était dessous. La caisse a presque tous les cubes. Le tapis est libre, au milieu. La nappe peut s'ouvrir ? Oui, maman. Raphaël pose la main sur le doudou. Le tissu est un peu rêche.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Un cube vert reste sur le tapis. Raphaël le glisse dans la caisse. Toc. Tu regardes bien dessous ? Oui, maman. La tour devient plus petite. Un bout de tapis reparaît. Encore un, tout doux. Le cube jaune va dans la caisse. Toc. Raphaël écarte un cube bas. Un coin de tissu gris. Mon doudou ! Le doudou était sous la tour. Il sent encore le lit. Raphaël le serre contre sa joue. Le tissu est chaud, tout doux. Te voilà, petit. Merci, tu l'as trouvé. Il était dessous. La caisse a presque tous les cubes. Le tapis est libre, au milieu. La nappe peut s'ouvrir, maintenant.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël refuse de prendre toute la pile. Il pose un genou au tapis. Un cube vert reste près de sa main. Je le mets tout seul. Il glisse le cube dans la &lt;emphasis level="moderate"&gt;caisse&lt;/emphasis&gt;. Toc. Le bois sent un peu la forêt. Tu regardes bien dessous ? Oui, maman. La tour devient plus petite. Un bout de tapis reparaît. Le cube jaune va dans la caisse. Toc. Je sors le reste, d'un coup ! Il tire trop fort sur un cube bas. Deux cubes retombent, comme un toit. Oh. Il ne reprend pas trop vite. Il écoute le salon, un instant. Sur la chaise, l'éclat de nappe brille. Il est là. Raphaël refuse de foncer. Il écarte un cube, lentement. Un coin de tissu gris. Mon doudou ! Le doudou était sous la tour. Il sent le tapis, un peu chaud. Raphaël le serre contre sa joue. Merci, Raphaël. Il était dessous. La caisse a presque tous les cubes. Le tapis est libre, au milieu. La nappe peut s'ouvrir ? Oui, maman. Raphaël pose la main sur le doudou. Le tissu est un peu rêche.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Léa a rangé. Les cubes sont dans la &lt;emphasis&gt;caisse&lt;/emphasis&gt;. Le tapis est libre. Maman est là.&lt;/slow&gt; [pause]</t>
+          <t>Raphaël refuse de prendre toute la pile. Il pose un genou au tapis. Un cube vert reste près de sa main. Je le mets tout seul. Il glisse le cube dans la &lt;emphasis&gt;caisse&lt;/emphasis&gt;. Toc. Le bois sent un peu la forêt. Tu regardes bien dessous ? Oui, maman. La tour devient plus petite. Un bout de tapis reparaît. Le cube jaune va dans la caisse. Toc. Je sors le reste, d'un coup ! Il tire trop fort sur un cube bas. Deux cubes retombent, comme un toit. Oh. Il ne reprend pas trop vite. Il écoute le salon, un instant. Sur la chaise, l'éclat de nappe brille. Il est là. Raphaël refuse de foncer. Il écarte un cube, lentement. Un coin de tissu gris. Mon doudou ! Le doudou était sous la tour. Il sent le tapis, un peu chaud. Raphaël le serre contre sa joue. Merci, Raphaël. Il était dessous. La caisse a presque tous les cubes. Le tapis est libre, au milieu. La nappe peut s'ouvrir ? Oui, maman. Raphaël pose la main sur le doudou. Le tissu est un peu rêche. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1646,7 +1661,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1654,10 +1669,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1687,23 +1702,23 @@
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1712,10 +1727,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1724,38 +1739,56 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_pose_un_cube_sans_foncer; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Un cube vert reste sur le tapis.
-narrateur|Raphaël le glisse dans la caisse.
+          <t>narrateur|Raphaël refuse de prendre toute la pile.
+narrateur|Il pose un genou au tapis.
+narrateur|Un cube vert reste près de sa main.
+enfant-m|Je le mets tout seul.
+narrateur|Il glisse le cube dans la caisse.
 narrateur|Toc.
+narrateur|Le bois sent un peu la forêt.
 maman|Tu regardes bien dessous ?
 enfant-m|Oui, maman.
 narrateur|La tour devient plus petite.
 narrateur|Un bout de tapis reparaît.
-papa|Encore un, tout doux.
 narrateur|Le cube jaune va dans la caisse.
 narrateur|Toc.
-narrateur|Raphaël écarte un cube bas.
+enfant-m|Je sors le reste, d'un coup !
+narrateur|Il tire trop fort sur un cube bas.
+narrateur|Deux cubes retombent, comme un toit.
+enfant-m|Oh.
+narrateur|Il ne reprend pas trop vite.
+narrateur|Il écoute le salon, un instant.
+narrateur|Sur la chaise, l'éclat de nappe brille.
+enfant-m|Il est là.
+narrateur|Raphaël refuse de foncer.
+narrateur|Il écarte un cube, lentement.
 narrateur|Un coin de tissu gris.
 enfant-m|Mon doudou !
 narrateur|Le doudou était sous la tour.
-narrateur|Il sent encore le lit.
+narrateur|Il sent le tapis, un peu chaud.
 narrateur|Raphaël le serre contre sa joue.
-narrateur|Le tissu est chaud, tout doux.
-maman|Te voilà, petit.
-papa|Merci, tu l'as trouvé.
+papa|Merci, Raphaël.
 enfant-m|Il était dessous.
 narrateur|La caisse a presque tous les cubes.
 narrateur|Le tapis est libre, au milieu.
-maman|La nappe peut s'ouvrir, maintenant.</t>
+maman|La nappe peut s'ouvrir ?
+enfant-m|Oui, maman.
+narrateur|Raphaël pose la main sur le doudou.
+narrateur|Le tissu est un peu rêche.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>caisse,bois</t>
         </is>
       </c>
     </row>
@@ -1782,17 +1815,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman déplie la nappe à carreaux. Raphaël tient un coin. Les carreaux sont rouges et blancs. La nappe est plate, enfin. Le vrai gâteau peut s'asseoir. Papa pose le plat chaud. La vanille remplit le salon. Le doudou a un carreau. Oui, le carreau rouge. Raphaël casse un bout tiède. La miette fond un peu. C'est bon, papa. On est bien, ici. Tu veux un peu d'eau ? Oui, maman. L'eau fait un petit bruit. Le soleil touche un carreau. Le doudou reste contre lui.</t>
+          <t>On déplie la nappe ? Maman déplie la nappe à carreaux. Raphaël tient un coin. Les carreaux sont rouges et blancs. Un cube oublié accroche le tissu. Je tire ! Raphaël s'arrête. Il refuse de foncer. Il recule le cube, lentement. La nappe se pose, plate. Le vrai gâteau peut s'asseoir. Papa pose le plat chaud. La vanille remplit le salon. Le doudou a un carreau. Oui, le carreau rouge. L'éclat de nappe tremble sur le rouge. Tu veux un peu d'eau ? Oui, papa. L'eau fait un petit bruit. Raphaël casse un bout tiède. La miette fond un peu. C'est bon, papa. On est bien, ici. Le doudou reste contre lui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Maman déplie la nappe à carreaux. Raphaël tient un coin. Les carreaux sont rouges et blancs. La nappe est plate, enfin. Le vrai gâteau peut s'asseoir. Papa pose le plat chaud. La vanille remplit le salon. Le doudou a un carreau. Oui, le carreau rouge. Raphaël casse un bout tiède. La miette fond un peu. C'est bon, papa. On est bien, ici. Tu veux un peu d'eau ? Oui, maman. L'eau fait un petit bruit. Le soleil touche un carreau. Le doudou reste contre lui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On déplie la &lt;emphasis level="moderate"&gt;nappe&lt;/emphasis&gt; ? Maman déplie la nappe à carreaux. Raphaël tient un coin. Les carreaux sont rouges et blancs. Un cube oublié accroche le tissu. Je tire ! Raphaël s'arrête. Il refuse de foncer. Il recule le cube, lentement. La nappe se pose, plate. Le vrai gâteau peut s'asseoir. Papa pose le plat chaud. La vanille remplit le salon. Le doudou a un carreau. Oui, le carreau rouge. L'éclat de nappe tremble sur le rouge. Tu veux un peu d'eau ? Oui, papa. L'eau fait un petit bruit. Raphaël casse un bout tiède. La miette fond un peu. C'est bon, papa. On est bien, ici. Le doudou reste contre lui.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Léa ferme la &lt;emphasis&gt;caisse&lt;/emphasis&gt;. Ça fait toc. Maman lui tend l'eau.&lt;/slow&gt; [pause]</t>
+          <t>On déplie la &lt;emphasis&gt;nappe&lt;/emphasis&gt; ? Maman déplie la nappe à carreaux. Raphaël tient un coin. Les carreaux sont rouges et blancs. Un cube oublié accroche le tissu. Je tire ! Raphaël s'arrête. Il refuse de foncer. Il recule le cube, lentement. La nappe se pose, plate. Le vrai gâteau peut s'asseoir. Papa pose le plat chaud. La vanille remplit le salon. Le doudou a un carreau. Oui, le carreau rouge. L'éclat de nappe tremble sur le rouge. Tu veux un peu d'eau ? Oui, papa. L'eau fait un petit bruit. Raphaël casse un bout tiède. La miette fond un peu. C'est bon, papa. On est bien, ici. Le doudou reste contre lui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1839,7 +1872,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1847,10 +1880,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1873,30 +1906,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>caisse</t>
+          <t>nappe</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1905,10 +1938,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1917,29 +1950,44 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_tirer_la_nappe; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman déplie la nappe à carreaux.
+          <t>papa|On déplie la nappe ?
+narrateur|Maman déplie la nappe à carreaux.
 narrateur|Raphaël tient un coin.
 narrateur|Les carreaux sont rouges et blancs.
-narrateur|La nappe est plate, enfin.
+narrateur|Un cube oublié accroche le tissu.
+enfant-m|Je tire !
+narrateur|Raphaël s'arrête.
+narrateur|Il refuse de foncer.
+narrateur|Il recule le cube, lentement.
+narrateur|La nappe se pose, plate.
 papa|Le vrai gâteau peut s'asseoir.
 narrateur|Papa pose le plat chaud.
 narrateur|La vanille remplit le salon.
 enfant-m|Le doudou a un carreau.
 maman|Oui, le carreau rouge.
+narrateur|L'éclat de nappe tremble sur le rouge.
+papa|Tu veux un peu d'eau ?
+enfant-m|Oui, papa.
+narrateur|L'eau fait un petit bruit.
 narrateur|Raphaël casse un bout tiède.
 narrateur|La miette fond un peu.
 enfant-m|C'est bon, papa.
-papa|On est bien, ici.
-maman|Tu veux un peu d'eau ?
-enfant-m|Oui, maman.
-narrateur|L'eau fait un petit bruit.
-narrateur|Le soleil touche un carreau.
+maman|On est bien, ici.
 narrateur|Le doudou reste contre lui.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>nappe,plat</t>
         </is>
       </c>
     </row>
@@ -1966,17 +2014,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a du gâteau. Un tout petit bout. Bravo, tu l'as retrouvé. La vanille reste dans l'air. Les carreaux sont chauds, maintenant.</t>
+          <t>Ils s'assoient près de la nappe tiède. La chaleur touche les joues de Raphaël. Le gâteau est là. Oui, tout chaud. Le doudou a un tout petit bout. Comme l'éclat de nappe, papa ! Tu le vois, toi ? Oui, sur le carreau rouge. Raphaël glisse le doudou sans se presser. Le tissu repose contre sa hanche. On le sent, maman. Tu le sens sur tes joues ? Oui, il est chaud. La vanille reste dans l'air. L'éclat de nappe tient sur le carreau.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a du gâteau. Un tout petit bout. Bravo, tu l'as retrouvé. La vanille reste dans l'air. Les carreaux sont chauds, maintenant.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils s'assoient près de la nappe tiède. La chaleur touche les joues de Raphaël. Le gâteau est là. Oui, tout chaud. Le doudou a un tout petit bout. Comme l'&lt;emphasis level="moderate"&gt;éclat de nappe&lt;/emphasis&gt;, papa ! Tu le vois, toi ? Oui, sur le carreau rouge. Raphaël glisse le doudou sans se presser. Le tissu repose contre sa hanche. On le sent, maman. Tu le sens sur tes joues ? Oui, il est chaud. La vanille reste dans l'air. L'éclat de nappe tient sur le carreau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils s'assoient près de la nappe tiède. La chaleur touche les joues de Raphaël. Le gâteau est là. Oui, tout chaud. Le doudou a un tout petit bout. Comme l'&lt;emphasis&gt;éclat de nappe&lt;/emphasis&gt;, papa ! Tu le vois, toi ? Oui, sur le carreau rouge. Raphaël glisse le doudou sans se presser. Le tissu repose contre sa hanche. On le sent, maman. Tu le sens sur tes joues ? Oui, il est chaud. La vanille reste dans l'air. L'éclat de nappe tient sur le carreau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2023,18 +2071,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2043,12 +2091,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2057,17 +2105,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de nappe</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2076,11 +2128,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2089,28 +2141,47 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_carreau; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|Le doudou a du gâteau.
-maman|Un tout petit bout.
-papa|Bravo, tu l'as retrouvé.
+          <t>narrateur|Ils s'assoient près de la nappe tiède.
+narrateur|La chaleur touche les joues de Raphaël.
+enfant-m|Le gâteau est là.
+maman|Oui, tout chaud.
+narrateur|Le doudou a un tout petit bout.
+enfant-m|Comme l'éclat de nappe, papa !
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur le carreau rouge.
+narrateur|Raphaël glisse le doudou sans se presser.
+narrateur|Le tissu repose contre sa hanche.
+enfant-m|On le sent, maman.
+maman|Tu le sens sur tes joues ?
+enfant-m|Oui, il est chaud.
 narrateur|La vanille reste dans l'air.
-narrateur|Les carreaux sont chauds, maintenant.</t>
+narrateur|L'éclat de nappe tient sur le carreau.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>gâteau,vanille</t>
         </is>
       </c>
     </row>
@@ -2131,7 +2202,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2195,6 +2266,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-019): polish ATOM-AUT.RAN.001-01 xlsx
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.RAN.001-01.xlsx
+++ b/stories/arbres/ATOM-AUT.RAN.001-01.xlsx
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La vanille arrive dans le salon, avant le gâteau. Un carré de buée s'ouvre sur la vitre. La cuillère en bois tape dans le bol. Le gâteau est bientôt prêt. Il sent bon, papa. Dans le salon, le tapis est épais. Une nappe à carreaux attend, pliée. Elle repose sur la chaise. Sur un carreau rouge, un éclat de nappe brille. Il est tout petit, maman. C'est un éclat de nappe. Le tissu sent un peu le savon. Raphaël, tu sens le gâteau ? Oui, papa. Je veux la tour, maintenant ! Pendant que le gâteau refroidit ? Oui, une tour haute. En ce moment, Raphaël saisit un cube. Le cube vert est lisse, un peu froid. Il le pose au milieu du tapis. Ça fait clic, tout petit. Puis un cube jaune. Ça fait clic, contre le vert. Le cube du haut, c'est le gâteau. Un gâteau de cubes ! Le doudou gris est au pied. Raphaël l'assoit contre la tour. Toi, tu goûtes avec nous. Elle est belle, ta tour. Raphaël veut un cube de plus. Il le pose trop vite. Un cube jaune glisse. La tour penche. Trois cubes tombent sur le doudou. Oh. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Où est mon doudou ? Sous la nappe, peut-être ? Il va vers la chaise. Il soulève un coin du tissu. L'éclat de nappe tremble, puis tient. Pas de tissu gris. Il n'est pas là. Près du canapé ? Sa main passe sous le coussin. Le coussin est moelleux. Le doudou n'est pas là. Il est perdu. Je prends tout, d'un coup ! Il saisit la pile trop vite. Les cubes glissent entre ses doigts. Le tapis disparaît sous les cubes. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes sous les cubes ?</t>
+          <t>La vanille arrive dans le salon, avant le gâteau. Un carré de buée s'ouvre sur la vitre. La cuillère en bois tape dans le bol. Le gâteau est bientôt prêt. Il sent bon, papa. Dans le salon, le tapis est épais. Une nappe à carreaux attend, pliée. Elle repose sur la chaise. Sur un carreau rouge, un éclat de nappe brille. Il est tout petit, maman. C'est le soleil sur le rouge. Le tissu sent un peu le savon. Raphaël, tu sens le gâteau ? Oui, papa. Je veux la tour, maintenant ! Pendant que le gâteau refroidit ? Oui, une tour haute. En ce moment, Raphaël saisit un cube. Le cube vert est lisse, un peu froid. Il le pose au milieu du tapis. Ça fait clic, tout petit. Puis un cube jaune. Ça fait clic, contre le vert. Le cube du haut, c'est le gâteau. Un gâteau de cubes ! Le doudou gris est au pied. Raphaël l'assoit contre la tour. Toi, tu goûtes avec nous. Elle est belle, ta tour. Raphaël veut un cube de plus. Il le pose trop vite. Un cube jaune glisse. La tour penche. Trois cubes tombent sur le doudou. Oh. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Où est mon doudou ? Sous la nappe, peut-être ? Il va vers la chaise. Il soulève un coin du tissu. L'éclat de nappe tremble, puis tient. Pas de tissu gris. Il n'est pas là. Près du canapé ? Sa main passe sous le coussin. Le coussin est moelleux. Le doudou n'est pas là. Il est perdu. Je prends tout, d'un coup ! Il saisit la pile trop vite. Les cubes glissent entre ses doigts. Le tapis disparaît sous les cubes. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes sous les cubes ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La vanille arrive dans le salon, avant le gâteau. Un carré de buée s'ouvre sur la vitre. La cuillère en bois tape dans le bol. Le gâteau est bientôt prêt. Il sent bon, papa. Dans le salon, le tapis est épais. Une nappe à carreaux attend, pliée. Elle repose sur la chaise. Sur un carreau rouge, un &lt;emphasis level="moderate"&gt;éclat de nappe&lt;/emphasis&gt; brille. Il est tout petit, maman. C'est un éclat de nappe. Le tissu sent un peu le savon. Raphaël, tu sens le gâteau ? Oui, papa. Je veux la tour, maintenant ! Pendant que le gâteau refroidit ? Oui, une tour haute. En ce moment, Raphaël saisit un cube. Le cube vert est lisse, un peu froid. Il le pose au milieu du tapis. Ça fait clic, tout petit. Puis un cube jaune. Ça fait clic, contre le vert. Le cube du haut, c'est le gâteau. Un gâteau de cubes ! Le doudou gris est au pied. Raphaël l'assoit contre la tour. Toi, tu goûtes avec nous. Elle est belle, ta tour. Raphaël veut un cube de plus. Il le pose trop vite. Un cube jaune glisse. La tour penche. Trois cubes tombent sur le doudou. Oh. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Où est mon doudou ? Sous la nappe, peut-être ? Il va vers la chaise. Il soulève un coin du tissu. L'éclat de nappe tremble, puis tient. Pas de tissu gris. Il n'est pas là. Près du canapé ? Sa main passe sous le coussin. Le coussin est moelleux. Le doudou n'est pas là. Il est perdu. Je prends tout, d'un coup ! Il saisit la pile trop vite. Les cubes glissent entre ses doigts. Le tapis disparaît sous les cubes. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes sous les cubes ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La vanille arrive dans le salon, avant le gâteau. Un carré de buée s'ouvre sur la vitre. La cuillère en bois tape dans le bol. Le gâteau est bientôt prêt. Il sent bon, papa. Dans le salon, le tapis est épais. Une nappe à carreaux attend, pliée. Elle repose sur la chaise. Sur un carreau rouge, un &lt;emphasis level="moderate"&gt;éclat de nappe&lt;/emphasis&gt; brille. Il est tout petit, maman. C'est le soleil sur le rouge. Le tissu sent un peu le savon. Raphaël, tu sens le gâteau ? Oui, papa. Je veux la tour, maintenant ! Pendant que le gâteau refroidit ? Oui, une tour haute. En ce moment, Raphaël saisit un cube. Le cube vert est lisse, un peu froid. Il le pose au milieu du tapis. Ça fait clic, tout petit. Puis un cube jaune. Ça fait clic, contre le vert. Le cube du haut, c'est le gâteau. Un gâteau de cubes ! Le doudou gris est au pied. Raphaël l'assoit contre la tour. Toi, tu goûtes avec nous. Elle est belle, ta tour. Raphaël veut un cube de plus. Il le pose trop vite. Un cube jaune glisse. La tour penche. Trois cubes tombent sur le doudou. Oh. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Où est mon doudou ? Sous la nappe, peut-être ? Il va vers la chaise. Il soulève un coin du tissu. L'éclat de nappe tremble, puis tient. Pas de tissu gris. Il n'est pas là. Près du canapé ? Sa main passe sous le coussin. Le coussin est moelleux. Le doudou n'est pas là. Il est perdu. Je prends tout, d'un coup ! Il saisit la pile trop vite. Les cubes glissent entre ses doigts. Le tapis disparaît sous les cubes. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes sous les cubes ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>La vanille arrive dans le salon, avant le gâteau. Un carré de buée s'ouvre sur la vitre. La cuillère en bois tape dans le bol. Le gâteau est bientôt prêt. Il sent bon, papa. Dans le salon, le tapis est épais. Une nappe à carreaux attend, pliée. Elle repose sur la chaise. Sur un carreau rouge, un &lt;emphasis&gt;éclat de nappe&lt;/emphasis&gt; brille. Il est tout petit, maman. C'est un éclat de nappe. Le tissu sent un peu le savon. Raphaël, tu sens le gâteau ? Oui, papa. Je veux la tour, maintenant ! Pendant que le gâteau refroidit ? Oui, une tour haute. En ce moment, Raphaël saisit un cube. Le cube vert est lisse, un peu froid. Il le pose au milieu du tapis. Ça fait clic, tout petit. Puis un cube jaune. Ça fait clic, contre le vert. Le cube du haut, c'est le gâteau. Un gâteau de cubes ! Le doudou gris est au pied. Raphaël l'assoit contre la tour. Toi, tu goûtes avec nous. Elle est belle, ta tour. Raphaël veut un cube de plus. Il le pose trop vite. Un cube jaune glisse. La tour penche. Trois cubes tombent sur le doudou. Oh. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Où est mon doudou ? Sous la nappe, peut-être ? Il va vers la chaise. Il soulève un coin du tissu. L'éclat de nappe tremble, puis tient. Pas de tissu gris. Il n'est pas là. Près du canapé ? Sa main passe sous le coussin. Le coussin est moelleux. Le doudou n'est pas là. Il est perdu. Je prends tout, d'un coup ! Il saisit la pile trop vite. Les cubes glissent entre ses doigts. Le tapis disparaît sous les cubes. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes sous les cubes ? [pause]</t>
+          <t>La vanille arrive dans le salon, avant le gâteau. Un carré de buée s'ouvre sur la vitre. La cuillère en bois tape dans le bol. Le gâteau est bientôt prêt. Il sent bon, papa. Dans le salon, le tapis est épais. Une nappe à carreaux attend, pliée. Elle repose sur la chaise. Sur un carreau rouge, un &lt;emphasis&gt;éclat de nappe&lt;/emphasis&gt; brille. Il est tout petit, maman. C'est le soleil sur le rouge. Le tissu sent un peu le savon. Raphaël, tu sens le gâteau ? Oui, papa. Je veux la tour, maintenant ! Pendant que le gâteau refroidit ? Oui, une tour haute. En ce moment, Raphaël saisit un cube. Le cube vert est lisse, un peu froid. Il le pose au milieu du tapis. Ça fait clic, tout petit. Puis un cube jaune. Ça fait clic, contre le vert. Le cube du haut, c'est le gâteau. Un gâteau de cubes ! Le doudou gris est au pied. Raphaël l'assoit contre la tour. Toi, tu goûtes avec nous. Elle est belle, ta tour. Raphaël veut un cube de plus. Il le pose trop vite. Un cube jaune glisse. La tour penche. Trois cubes tombent sur le doudou. Oh. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Où est mon doudou ? Sous la nappe, peut-être ? Il va vers la chaise. Il soulève un coin du tissu. L'éclat de nappe tremble, puis tient. Pas de tissu gris. Il n'est pas là. Près du canapé ? Sa main passe sous le coussin. Le coussin est moelleux. Le doudou n'est pas là. Il est perdu. Je prends tout, d'un coup ! Il saisit la pile trop vite. Les cubes glissent entre ses doigts. Le tapis disparaît sous les cubes. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes sous les cubes ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1338,7 +1338,7 @@
 narrateur|Elle repose sur la chaise.
 narrateur|Sur un carreau rouge, un éclat de nappe brille.
 enfant-m|Il est tout petit, maman.
-maman|C'est un éclat de nappe.
+maman|C'est le soleil sur le rouge.
 narrateur|Le tissu sent un peu le savon.
 papa|Raphaël, tu sens le gâteau ?
 enfant-m|Oui, papa.
@@ -1815,17 +1815,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On déplie la nappe ? Maman déplie la nappe à carreaux. Raphaël tient un coin. Les carreaux sont rouges et blancs. Un cube oublié accroche le tissu. Je tire ! Raphaël s'arrête. Il refuse de foncer. Il recule le cube, lentement. La nappe se pose, plate. Le vrai gâteau peut s'asseoir. Papa pose le plat chaud. La vanille remplit le salon. Le doudou a un carreau. Oui, le carreau rouge. L'éclat de nappe tremble sur le rouge. Tu veux un peu d'eau ? Oui, papa. L'eau fait un petit bruit. Raphaël casse un bout tiède. La miette fond un peu. C'est bon, papa. On est bien, ici. Le doudou reste contre lui.</t>
+          <t>On déplie la nappe ? Maman déplie la nappe à carreaux. Raphaël tient un coin. Les carreaux sont rouges et blancs. Un cube oublié accroche le tissu. Je tire ! Raphaël s'arrête. Il refuse de foncer. Il recule le cube, lentement. La nappe se pose, plate. Le vrai gâteau peut s'asseoir. Papa pose le plat chaud. La vanille remplit le salon. Le doudou a un carreau. Oui, le carreau rouge. Le carreau rouge tremble un peu. Tu veux un peu d'eau ? Oui, papa. L'eau fait un petit bruit. Raphaël casse un bout tiède. La miette fond un peu. C'est bon, papa. On est bien, ici. Le doudou reste contre lui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On déplie la &lt;emphasis level="moderate"&gt;nappe&lt;/emphasis&gt; ? Maman déplie la nappe à carreaux. Raphaël tient un coin. Les carreaux sont rouges et blancs. Un cube oublié accroche le tissu. Je tire ! Raphaël s'arrête. Il refuse de foncer. Il recule le cube, lentement. La nappe se pose, plate. Le vrai gâteau peut s'asseoir. Papa pose le plat chaud. La vanille remplit le salon. Le doudou a un carreau. Oui, le carreau rouge. L'éclat de nappe tremble sur le rouge. Tu veux un peu d'eau ? Oui, papa. L'eau fait un petit bruit. Raphaël casse un bout tiède. La miette fond un peu. C'est bon, papa. On est bien, ici. Le doudou reste contre lui.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On déplie la &lt;emphasis level="moderate"&gt;nappe&lt;/emphasis&gt; ? Maman déplie la nappe à carreaux. Raphaël tient un coin. Les carreaux sont rouges et blancs. Un cube oublié accroche le tissu. Je tire ! Raphaël s'arrête. Il refuse de foncer. Il recule le cube, lentement. La nappe se pose, plate. Le vrai gâteau peut s'asseoir. Papa pose le plat chaud. La vanille remplit le salon. Le doudou a un carreau. Oui, le carreau rouge. Le carreau rouge tremble un peu. Tu veux un peu d'eau ? Oui, papa. L'eau fait un petit bruit. Raphaël casse un bout tiède. La miette fond un peu. C'est bon, papa. On est bien, ici. Le doudou reste contre lui.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>On déplie la &lt;emphasis&gt;nappe&lt;/emphasis&gt; ? Maman déplie la nappe à carreaux. Raphaël tient un coin. Les carreaux sont rouges et blancs. Un cube oublié accroche le tissu. Je tire ! Raphaël s'arrête. Il refuse de foncer. Il recule le cube, lentement. La nappe se pose, plate. Le vrai gâteau peut s'asseoir. Papa pose le plat chaud. La vanille remplit le salon. Le doudou a un carreau. Oui, le carreau rouge. L'éclat de nappe tremble sur le rouge. Tu veux un peu d'eau ? Oui, papa. L'eau fait un petit bruit. Raphaël casse un bout tiède. La miette fond un peu. C'est bon, papa. On est bien, ici. Le doudou reste contre lui. [pause]</t>
+          <t>On déplie la &lt;emphasis&gt;nappe&lt;/emphasis&gt; ? Maman déplie la nappe à carreaux. Raphaël tient un coin. Les carreaux sont rouges et blancs. Un cube oublié accroche le tissu. Je tire ! Raphaël s'arrête. Il refuse de foncer. Il recule le cube, lentement. La nappe se pose, plate. Le vrai gâteau peut s'asseoir. Papa pose le plat chaud. La vanille remplit le salon. Le doudou a un carreau. Oui, le carreau rouge. Le carreau rouge tremble un peu. Tu veux un peu d'eau ? Oui, papa. L'eau fait un petit bruit. Raphaël casse un bout tiède. La miette fond un peu. C'est bon, papa. On est bien, ici. Le doudou reste contre lui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1974,7 +1974,7 @@
 narrateur|La vanille remplit le salon.
 enfant-m|Le doudou a un carreau.
 maman|Oui, le carreau rouge.
-narrateur|L'éclat de nappe tremble sur le rouge.
+narrateur|Le carreau rouge tremble un peu.
 papa|Tu veux un peu d'eau ?
 enfant-m|Oui, papa.
 narrateur|L'eau fait un petit bruit.
@@ -2014,17 +2014,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Ils s'assoient près de la nappe tiède. La chaleur touche les joues de Raphaël. Le gâteau est là. Oui, tout chaud. Le doudou a un tout petit bout. Comme l'éclat de nappe, papa ! Tu le vois, toi ? Oui, sur le carreau rouge. Raphaël glisse le doudou sans se presser. Le tissu repose contre sa hanche. On le sent, maman. Tu le sens sur tes joues ? Oui, il est chaud. La vanille reste dans l'air. L'éclat de nappe tient sur le carreau.</t>
+          <t>Ils s'assoient près de la nappe tiède. La chaleur touche les joues de Raphaël. Le gâteau est là. Oui, tout chaud. Le doudou a un tout petit bout. Comme sur la chaise, papa ! Tu le vois, toi ? Oui, sur le carreau rouge. Raphaël glisse le doudou sans se presser. Le tissu repose contre sa hanche. On le sent, maman. Tu le sens sur tes joues ? Oui, il est chaud. La vanille reste dans l'air. L'éclat de nappe tient sur le carreau.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils s'assoient près de la nappe tiède. La chaleur touche les joues de Raphaël. Le gâteau est là. Oui, tout chaud. Le doudou a un tout petit bout. Comme l'&lt;emphasis level="moderate"&gt;éclat de nappe&lt;/emphasis&gt;, papa ! Tu le vois, toi ? Oui, sur le carreau rouge. Raphaël glisse le doudou sans se presser. Le tissu repose contre sa hanche. On le sent, maman. Tu le sens sur tes joues ? Oui, il est chaud. La vanille reste dans l'air. L'éclat de nappe tient sur le carreau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils s'assoient près de la nappe tiède. La chaleur touche les joues de Raphaël. Le gâteau est là. Oui, tout chaud. Le doudou a un tout petit bout. Comme sur la chaise, papa ! Tu le vois, toi ? Oui, sur le carreau rouge. Raphaël glisse le doudou sans se presser. Le tissu repose contre sa hanche. On le sent, maman. Tu le sens sur tes joues ? Oui, il est chaud. La vanille reste dans l'air. L'&lt;emphasis level="moderate"&gt;éclat de nappe&lt;/emphasis&gt; tient sur le carreau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils s'assoient près de la nappe tiède. La chaleur touche les joues de Raphaël. Le gâteau est là. Oui, tout chaud. Le doudou a un tout petit bout. Comme l'&lt;emphasis&gt;éclat de nappe&lt;/emphasis&gt;, papa ! Tu le vois, toi ? Oui, sur le carreau rouge. Raphaël glisse le doudou sans se presser. Le tissu repose contre sa hanche. On le sent, maman. Tu le sens sur tes joues ? Oui, il est chaud. La vanille reste dans l'air. L'éclat de nappe tient sur le carreau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils s'assoient près de la nappe tiède. La chaleur touche les joues de Raphaël. Le gâteau est là. Oui, tout chaud. Le doudou a un tout petit bout. Comme sur la chaise, papa ! Tu le vois, toi ? Oui, sur le carreau rouge. Raphaël glisse le doudou sans se presser. Le tissu repose contre sa hanche. On le sent, maman. Tu le sens sur tes joues ? Oui, il est chaud. La vanille reste dans l'air. L'&lt;emphasis&gt;éclat de nappe&lt;/emphasis&gt; tient sur le carreau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2167,7 +2167,7 @@
 enfant-m|Le gâteau est là.
 maman|Oui, tout chaud.
 narrateur|Le doudou a un tout petit bout.
-enfant-m|Comme l'éclat de nappe, papa !
+enfant-m|Comme sur la chaise, papa !
 papa|Tu le vois, toi ?
 enfant-m|Oui, sur le carreau rouge.
 narrateur|Raphaël glisse le doudou sans se presser.
@@ -2202,7 +2202,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2273,6 +2273,13 @@
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>